<commit_message>
add order column and generations
</commit_message>
<xml_diff>
--- a/examples/input.example.xlsx
+++ b/examples/input.example.xlsx
@@ -46,8 +46,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -122,6 +123,26 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Historical Bloodlines</author>
+  </authors>
+  <commentList>
+    <comment ref="H2" authorId="0" shapeId="0">
+      <text>
+        <t>Необязательное положительное целое число.</t>
+      </text>
+    </comment>
+    <comment ref="I2" authorId="0" shapeId="0">
+      <text>
+        <t>Меньшее число располагается левее. Рекомендуемый шаг: 10.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -413,8 +434,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -464,6 +489,16 @@
           <t>Брак</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Поколение</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Порядок в поколении</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -489,6 +524,12 @@
           <t>Жоффруа Плантагенет</t>
         </is>
       </c>
+      <c r="H3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -514,6 +555,12 @@
           <t>Матильда</t>
         </is>
       </c>
+      <c r="H4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -545,6 +592,12 @@
           <t>Алиенора Аквитанская</t>
         </is>
       </c>
+      <c r="H5" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -570,6 +623,12 @@
           <t>Генрих II</t>
         </is>
       </c>
+      <c r="H6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -591,6 +650,12 @@
       <c r="E7" t="n">
         <v>1199</v>
       </c>
+      <c r="H7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -617,6 +682,12 @@
           <t>Генрих III</t>
         </is>
       </c>
+      <c r="H8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -638,8 +709,20 @@
       <c r="E9" t="n">
         <v>1272</v>
       </c>
+      <c r="H9" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="H3:I9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>